<commit_message>
fix : import template student
</commit_message>
<xml_diff>
--- a/school-management/src/main/resources/templates/student_import_template_vn 1.xlsx
+++ b/school-management/src/main/resources/templates/student_import_template_vn 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School\School-Management-System\school-management\src\main\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95085E53-05CE-48A8-92A3-C89B765EFE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DE0091-D18A-4F1F-8D62-A11FC23ED11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25305" yWindow="3495" windowWidth="21600" windowHeight="11055" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HuongDan" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="110">
   <si>
     <t>HƯỚNG DẪN IMPORT DANH SÁCH HỌC SINH</t>
   </si>
@@ -365,6 +365,10 @@
   </si>
   <si>
     <t>cuong.tv@example.com</t>
+  </si>
+  <si>
+    <t>CCCD
+(nation_id)</t>
   </si>
 </sst>
 </file>
@@ -457,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
@@ -488,6 +492,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1181,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1196,9 +1210,10 @@
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="16" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>57</v>
       </c>
@@ -1235,8 +1250,11 @@
       <c r="L1" s="5" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M1" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="6"/>
       <c r="B2" s="6" t="s">
         <v>69</v>
@@ -1271,8 +1289,11 @@
       <c r="L2" s="6" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M2" s="14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1309,8 +1330,11 @@
       <c r="L3" s="9" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M3" s="12">
+        <v>2799008128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1345,8 +1369,9 @@
       <c r="L4" s="9" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M4" s="12"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1375,6 +1400,9 @@
         <v>80</v>
       </c>
       <c r="L5" s="9"/>
+      <c r="M5" s="12">
+        <v>912000111</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -1386,7 +1414,7 @@
     </dataValidation>
     <dataValidation type="date" errorTitle="Ngày sinh không hợp lệ" error="Phải là ngày hợp lệ (YYYY-MM-DD)" sqref="D3:D1000" xr:uid="{00000000-0002-0000-0100-000002000000}"/>
     <dataValidation type="date" allowBlank="1" sqref="L3:L1000" xr:uid="{00000000-0002-0000-0100-000003000000}"/>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" sqref="F3:F1000" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" sqref="F3:F1000 M3:M1000" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>15</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>